<commit_message>
fix bug completion and equipment
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportCompletionRateErrorTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportCompletionRateErrorTemplate.xlsx
@@ -40,7 +40,7 @@
     <numFmt numFmtId="165" formatCode="0.00%"/>
     <numFmt numFmtId="166" formatCode="@"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -63,13 +63,13 @@
       <family val="0"/>
     </font>
     <font>
-      <sz val="14"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="14"/>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color rgb="FFFF0000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -86,6 +86,12 @@
       <b val="true"/>
       <sz val="14"/>
       <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
@@ -133,7 +139,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -159,6 +165,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -180,14 +190,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="17.35" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="22.79"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="7" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
fix calculate report external equality and change template completion rate
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportCompletionRateErrorTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportCompletionRateErrorTemplate.xlsx
@@ -77,14 +77,14 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="14"/>
+      <sz val="13"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="14"/>
+      <sz val="13"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -190,7 +190,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.43"/>

</xml_diff>